<commit_message>
fix: align prediction CSVs with Article 1 Table 3 definitive variants and harmonize versions in methods description form
</commit_message>
<xml_diff>
--- a/track1_variant_identification/manuscript_and_report/methods_description_form.xlsx
+++ b/track1_variant_identification/manuscript_and_report/methods_description_form.xlsx
@@ -626,7 +626,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Public reference panels: GRCh38/hg38 human reference genome, gnomAD v4.0 population allele frequencies, ClinVar (2026 release), OMIM, Ensembl release 112, 1000 Genomes Project Phase 3, STRING v12.0 interaction database, and my comprehensive global systematic meta-analysis of 158 peer-reviewed MVA cohort studies (1988–2026) consolidated from PubMed/MEDLINE.</t>
+          <t>Public reference panels: GRCh38/hg38 human reference genome, gnomAD v4.1 population allele frequencies, ClinVar (2026 release), OMIM, Ensembl release 112, 1000 Genomes Project Phase 3, STRING v12.0 interaction database, and my comprehensive global systematic meta-analysis of 158 peer-reviewed MVA cohort studies (1988–2026) consolidated from PubMed/MEDLINE.</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
           <t>Method Abstract:
 Mosaic Variegated Aneuploidy (MVA) syndrome is an ultra-rare, life-threatening chromosomal instability disorder defined by constitutional mosaic aneuploidies, premature chromatid separation (PCS), severe progressive microcephaly, profound intrauterine growth restriction, intractable medullary nephrocalcinosis, and heightened predisposition to embryonal malignancies. As an internal medicine specialist, I approached this challenge by integrating clinical bedside semiology with advanced computational genomics to dissect the patient's multi-system phenotype beyond chromosome enumeration.
 Methodological Detail:
-Index proband whole-genome sequencing data (85.0 GB raw paired-end FASTQ, 229,442,288 reads, 32.4x mean genomic depth) underwent rigorous automated quality filtration via fastp (v0.23.4, Q30 &gt; 94.0%, low optical duplication &lt; 8.0%), alignment against GRCh38/hg38 with BWA-MEM2, and consensus dual-caller variant identification using Google DeepVariant (v1.6.1) and GATK4 HaplotypeCaller. To score and rank filtered alleles without heuristic bias, I engineered a calibrated trimodal Integrated Pathogenicity Index (IPI, scale 0.0–1.0) uniting: (1) 3D structural protein folding perturbations and thermodynamic stability (ΔΔGfold) via AlphaMissense; (2) 16 kb long-range chromatin accessibility, transcription factor binding, and splice disruption via AlphaGenome; and (3) zero-shot evolutionary conservation constraint and delta log-likelihood ratio (DeltaLLR) via Evo 2 (7B biological foundation model trained across 300 billion tokens spanning 500 million years of eukaryotic evolution). The pipeline directly integrates my comprehensive global meta-analysis synthesizing 158 clinical studies (138 cohorts, 1988–2026).
+Index proband whole-genome sequencing data (85.0 GB raw paired-end FASTQ, 229,442,288 reads, 32.4x mean genomic depth) underwent rigorous automated quality filtration via fastp (v0.23.4, Q30 &gt; 94.0%, low optical duplication &lt; 8.0%), alignment against GRCh38/hg38 with BWA-MEM2, and consensus dual-caller variant identification using Google DeepVariant (v1.6.0) and GATK4 HaplotypeCaller. To score and rank filtered alleles without heuristic bias, I engineered a calibrated trimodal Integrated Pathogenicity Index (IPI, scale 0.0–1.0) uniting: (1) 3D structural protein folding perturbations and thermodynamic stability (ΔΔGfold) via AlphaMissense; (2) 16 kb long-range chromatin accessibility, transcription factor binding, and splice disruption via AlphaGenome; and (3) zero-shot evolutionary conservation constraint and delta log-likelihood ratio (DeltaLLR) via Evo 2 (7B biological foundation model trained across 300 billion tokens spanning 500 million years of eukaryotic evolution). The pipeline directly integrates my comprehensive global meta-analysis synthesizing 158 clinical studies (138 cohorts, 1988–2026).
 Strengths:
 1. Unified Multimodal Resolution: Bridges deep non-coding regulatory impact, structural protein physics, and long-range phylogenetic conservation into a single, mathematically calibrated index (IPI).
 2. Discovered Novel Dual Pathophysiology: Successfully uncovered and validated the genetic driver of congenital medullary nephrocalcinosis—a homozygous frameshift insertion in the zinc-finger ZF2 domain of WT1 (chr11:32408514_dupA, p.Arg394fs, IPI: 0.7256)—co-segregating with canonical SAC mitotic spindle collapse driven by compound heterozygous BUB1B (p.Arg407Ter, IPI: 0.7894) and heterozygous kinetic motor destabilization in CENPE (p.Arg1079Gln, IPI: 0.8016).
@@ -767,7 +767,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>De novo precision chemogenomics, targeted senolysis, and systems-biology reverse engineering across six mechanistic axes: (1) Synthetic lethality targeting aneuploid tumor cells via WEE1/PKMYT1 inhibitors (MVA-SYN-001/005); (2) Platelet-sparing targeted senolysis via chimeric BCL-xL / Cereblon PROTACs (MVA-SEN-005 / MVA-PRO-01) protecting anucleated platelets; (3) Allosteric mecano-chemical stabilization of CENPE Kinesin-7 motor (MVA-CEN-009); (4) Neuroprotective inhibition of sterile microglial neuroinflammation via CNS-penetrant STING Cys91 antagonists (MVA-STING-013); (5) Renal tubular senolysis and thiazide/citrate synergy against medullary nephrocalcinosis; and (6) Bio-inspired Ambystoma mexicanum (Axolotl) amphipathic anticancer peptides (MVA-AMP-01, 12, 13; P1, P12, P13) inducing selective Caspase-3/7 apoptosis, reactivating SFN, RB1, BRCA1/2, and suppressing SASP cytokines IL6 and MMP2. Coupled with nonlinear Lie-derivative observability and a 4-pillar DSB-free curative roadmap (Adenine Base Editing, Prime Editing, SORT-LNPs).</t>
+          <t>De novo precision chemogenomics, targeted senolysis, and systems-biology reverse engineering across six mechanistic axes: (1) Synthetic lethality targeting aneuploid tumor cells via WEE1/PKMYT1 inhibitors (MVA-SYN-001/005); (2) Platelet-sparing targeted senolysis via chimeric BCL-xL / Cereblon PROTACs (MVA-SEN-005 / MVA-PRO-01) protecting anucleated platelets; (3) Allosteric mechanochemical stabilization of CENPE Kinesin-7 motor (MVA-CEN-009); (4) Neuroprotective inhibition of sterile microglial neuroinflammation via CNS-penetrant STING Cys91 antagonists (MVA-STING-013); (5) Renal tubular senolysis and thiazide/citrate synergy against medullary nephrocalcinosis; and (6) Bio-inspired Ambystoma mexicanum (Axolotl) amphipathic anticancer peptides (MVA-AMP-01, 12, 13; P1, P12, P13) inducing selective Caspase-3/7 apoptosis, reactivating SFN, RB1, BRCA1/2, and suppressing SASP cytokines IL6 and MMP2. Coupled with nonlinear Lie-derivative observability and a 4-pillar DSB-free curative roadmap (Adenine Base Editing, Prime Editing, SORT-LNPs).</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ChEMBL v33, PubChem, PDB (Protein Data Bank), AlphaFold Protein Structure Database, cBioPortal, Human Protein Atlas, CAMPR3 antimicrobial peptide database, and PubMed literature.</t>
+          <t>ChEMBL v34, PubChem, PDB (Protein Data Bank), AlphaFold Protein Structure Database, cBioPortal, Human Protein Atlas, CAMPR3 antimicrobial peptide database, and PubMed literature.</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Mechanism characterization: Causal biallelic BUB1B/CENPE mutations cause loss-of-function (LoF) in the Mitotic Checkpoint Complex (MCC), leading to premature sister chromatid separation, lagging chromosomes, and high rates of aneuploidy (PCS trait). The cellular consequence is dual: (A) In proliferating embryonic cells, chromosomal catastrophe triggers p53-dependent senescence or neoplastic transformation (Rhabdomyosarcoma/Wilms tumor); (B) Chronic micronuclei rupture releases double-stranded DNA into the cytosol, activating the cGAS-STING-TBK1-IRF3 axis, driving sterile neuroinflammation and SASP. Simultaneously, homozygous WT1 duplication impairs podocyte slit-diaphragm maintenance and dysregulates renal tubular TRPV5/Claudin-16 expression, causing medullary nephrocalcinosis.</t>
+          <t>Mechanism characterization: Causal biallelic BUB1B/CENPE mutations cause loss-of-function (LoF) in the Mitotic Checkpoint Complex (MCC), leading to premature sister chromatid separation, lagging chromosomes, and high rates of aneuploidy (PCS trait). The cellular consequence is dual: (A) In proliferating embryonic cells, chromosomal catastrophe triggers p53-dependent senescence or neoplastic transformation (Rhabdomyosarcoma/Wilms tumor); (B) Chronic micronuclei rupture releases double-stranded DNA into the cytosol, activating the cGAS-STING-TBK1-IRF3 axis, driving sterile neuroinflammation and SASP. Simultaneously, homozygous WT1 frameshift insertion (c.1180dupA, p.Arg394fs) impairs podocyte slit-diaphragm maintenance and dysregulates renal tubular TRPV5 and calbindin-D28k expression, causing medullary nephrocalcinosis.</t>
         </is>
       </c>
     </row>

</xml_diff>